<commit_message>
feat: update phase 5
</commit_message>
<xml_diff>
--- a/projects/mini-rally/07_Test Business/BUSINESS_E2E_TEST_TRACKER.xlsx
+++ b/projects/mini-rally/07_Test Business/BUSINESS_E2E_TEST_TRACKER.xlsx
@@ -294,7 +294,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="BusinessExecutionLog" displayName="BusinessExecutionLog" ref="A4:J35" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="BusinessExecutionLog" displayName="BusinessExecutionLog" ref="A4:J43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Execution ID"/>
     <x:tableColumn id="2" name="Step ID"/>
@@ -312,7 +312,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="BusinessGapLog" displayName="BusinessGapLog" ref="A4:M20" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="BusinessGapLog" displayName="BusinessGapLog" ref="A4:M28" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="13">
     <x:tableColumn id="1" name="Gap ID"/>
     <x:tableColumn id="2" name="Step ID"/>
@@ -586,7 +586,7 @@
       </x:c>
       <x:c r="B5" s="45" t="n">
         <x:f>COUNTIF('E2E Steps'!$I$5:$I$50,"Passed")</x:f>
-        <x:v>2</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D5" s="38"/>
       <x:c r="E5" s="39"/>
@@ -600,7 +600,7 @@
       </x:c>
       <x:c r="B6" s="45" t="n">
         <x:f>COUNTIF('E2E Steps'!$I$5:$I$50,"Failed")</x:f>
-        <x:v>1</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D6" s="38"/>
       <x:c r="E6" s="39"/>
@@ -614,7 +614,7 @@
       </x:c>
       <x:c r="B7" s="45" t="n">
         <x:f>COUNTIF('E2E Steps'!$I$5:$I$50,"Blocked")</x:f>
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D7" s="38"/>
       <x:c r="E7" s="39"/>
@@ -656,7 +656,7 @@
       </x:c>
       <x:c r="B10" s="45" t="n">
         <x:f>COUNTIF('E2E Steps'!$I$5:$I$50,"Not Started")</x:f>
-        <x:v>5</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="D10" s="38"/>
       <x:c r="E10" s="39"/>
@@ -670,7 +670,7 @@
       </x:c>
       <x:c r="B11" s="45" t="n">
         <x:f>COUNTA('Gap Log'!$A$5:$A$100)</x:f>
-        <x:v>16</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="D11" s="41"/>
       <x:c r="E11" s="42"/>
@@ -1177,19 +1177,23 @@
         <x:v>Task Dashboard/Detail</x:v>
       </x:c>
       <x:c r="I13" s="46" t="str">
-        <x:v>Blocked</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="J13" s="46" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="K13" s="46" t="str">
-        <x:v>TA-01; TA-02</x:v>
+        <x:v>TA-01 (TA-6); TA-02 (TA-7) -&gt; WI-01 (US-9)</x:v>
       </x:c>
       <x:c r="L13" s="46" t="str">
-        <x:v>Not executed. DevInt was turned off after the E2E-07 confirmation; resume from this checkpoint when the environment is available.</x:v>
-      </x:c>
-      <x:c r="M13" s="46" t="str"/>
-      <x:c r="N13" s="46" t="str"/>
+        <x:v>Re-run 2026-07-20 after DevInt reseed (TA-8/TA-9/US-12 wiped; recreated TA-6/TA-7 under US-9). On TA-6 set To Do=3 and logged Actual=2h via Task Detail; Estimate stayed blank instead of deriving 5. US-9 Task Roll-up read Estimate 4 / To Do 3 / Actual 2, so Total Estimate 4 != To Do 3 + Actual 2 = 5. Estimate is still an independent editable field (Add Task modal too). Actual is captured as a Time Logs entry-sum, not a manual actual_hours field. Completing a Task also zeroes its To Do. DEV-012 (badge shows 0) and DEV-014 (no inline edit) still reproduce. Positive: Task create and Task Detail routing now work.</x:v>
+      </x:c>
+      <x:c r="M13" s="46" t="str">
+        <x:v>DEV-013; DEV-015; DEV-016</x:v>
+      </x:c>
+      <x:c r="N13" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
       <x:c r="O13" s="47" t="n">
         <x:v>46223</x:v>
       </x:c>
@@ -1220,18 +1224,26 @@
         <x:v>Task Dashboard/Detail</x:v>
       </x:c>
       <x:c r="I14" s="46" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="J14" s="46" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="K14" s="46" t="str">
-        <x:v>TA-01; TA-02 -&gt; WI-01</x:v>
-      </x:c>
-      <x:c r="L14" s="46" t="str"/>
-      <x:c r="M14" s="46" t="str"/>
-      <x:c r="N14" s="46" t="str"/>
-      <x:c r="O14" s="47"/>
+        <x:v>TA-01 (TA-6); TA-02 (TA-7) -&gt; WI-01 (US-9)</x:v>
+      </x:c>
+      <x:c r="L14" s="46" t="str">
+        <x:v>Partial. Completing only TA-6 (1 of 2) left US-9 at Defined (correct). Completing TA-7 as well auto-changed US-9 Schedule State to Completed - auto-complete works. But US-9 Flow State stayed Defined, so Schedule and Flow did not mirror and the parent is not fully Completed per BR-WI-01 / TASK-FR-016. Task Detail also exposes Schedule State + Flow State instead of a single Task State.</x:v>
+      </x:c>
+      <x:c r="M14" s="46" t="str">
+        <x:v>DEV-016; DEV-017</x:v>
+      </x:c>
+      <x:c r="N14" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="O14" s="47" t="n">
+        <x:v>46223</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="66" customHeight="1">
       <x:c r="A15" s="46" t="str">
@@ -1259,18 +1271,26 @@
         <x:v>Task Dashboard/Detail</x:v>
       </x:c>
       <x:c r="I15" s="46" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="J15" s="46" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="K15" s="46" t="str">
-        <x:v>TA-01 -&gt; WI-01</x:v>
-      </x:c>
-      <x:c r="L15" s="46" t="str"/>
-      <x:c r="M15" s="46" t="str"/>
-      <x:c r="N15" s="46" t="str"/>
-      <x:c r="O15" s="47"/>
+        <x:v>TA-01 (TA-6) -&gt; WI-01 (US-9)</x:v>
+      </x:c>
+      <x:c r="L15" s="46" t="str">
+        <x:v>Reopened TA-6 from Completed to In Progress; the Task change persisted after reload. US-9 stayed Completed and did NOT auto-roll-back to In-Progress. The reopen -&gt; In-Progress rule (BR-TASK-02) is not implemented; the auto roll-up is one-way only.</x:v>
+      </x:c>
+      <x:c r="M15" s="46" t="str">
+        <x:v>DEV-016; DEV-018</x:v>
+      </x:c>
+      <x:c r="N15" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="O15" s="47" t="n">
+        <x:v>46223</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="66" customHeight="1">
       <x:c r="A16" s="46" t="str">
@@ -1298,18 +1318,26 @@
         <x:v>Backlog; Work Item Detail; Iteration Status</x:v>
       </x:c>
       <x:c r="I16" s="46" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="J16" s="46" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="K16" s="46" t="str">
-        <x:v>WI-01</x:v>
-      </x:c>
-      <x:c r="L16" s="46" t="str"/>
-      <x:c r="M16" s="46" t="str"/>
-      <x:c r="N16" s="46" t="str"/>
-      <x:c r="O16" s="47"/>
+        <x:v>US-7 / US-9 (probe)</x:v>
+      </x:c>
+      <x:c r="L16" s="46" t="str">
+        <x:v>Tested on US-7/US-9. Schedule State has 6 buttons (Idea..Release) but labels In Progress not In-Progress; Flow State dropdown has only 4 options (Defined/In Progress/Completed/Accepted), missing Idea and Release. Schedule&lt;-&gt;Flow do NOT mirror either way: Schedule=In Progress left Flow Defined; Flow=Completed left Schedule In Progress. US-7 reverted to Defined/Defined.</x:v>
+      </x:c>
+      <x:c r="M16" s="46" t="str">
+        <x:v>DEV-020</x:v>
+      </x:c>
+      <x:c r="N16" s="46" t="str">
+        <x:v>notes/E2E-11-13-STATUS-ITERATION.md</x:v>
+      </x:c>
+      <x:c r="O16" s="47" t="n">
+        <x:v>46223</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="66" customHeight="1">
       <x:c r="A17" s="46" t="str">
@@ -1337,18 +1365,26 @@
         <x:v>/iteration-status; /timeboxes</x:v>
       </x:c>
       <x:c r="I17" s="46" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="J17" s="46" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="K17" s="46" t="str">
-        <x:v>IT-01</x:v>
-      </x:c>
-      <x:c r="L17" s="46" t="str"/>
-      <x:c r="M17" s="46" t="str"/>
-      <x:c r="N17" s="46" t="str"/>
-      <x:c r="O17" s="47"/>
+        <x:v>IT-01 (Sprint 26.2); US-7; US-9</x:v>
+      </x:c>
+      <x:c r="L17" s="46" t="str">
+        <x:v>Set US-7 and US-9 (both Sprint 26.2 items) Schedule State = Accepted. Iteration Status ACCEPTED tile = 100% (13 of 13 pts) and iteration detail ACCEPTED 100% of committed, but Sprint 26.2 State stayed Planning in Timeboxes - did NOT auto-change to Accepted (BR-IT-02). Accepted metric correct; only the auto state transition is missing.</x:v>
+      </x:c>
+      <x:c r="M17" s="46" t="str">
+        <x:v>DEV-021</x:v>
+      </x:c>
+      <x:c r="N17" s="46" t="str">
+        <x:v>notes/E2E-11-13-STATUS-ITERATION.md</x:v>
+      </x:c>
+      <x:c r="O17" s="47" t="n">
+        <x:v>46223</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="66" customHeight="1">
       <x:c r="A18" s="46" t="str">
@@ -1376,18 +1412,26 @@
         <x:v>/timeboxes; /backlog</x:v>
       </x:c>
       <x:c r="I18" s="46" t="str">
-        <x:v>Not Started</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="J18" s="46" t="str">
-        <x:v>Pending</x:v>
+        <x:v>Confirmed</x:v>
       </x:c>
       <x:c r="K18" s="46" t="str">
-        <x:v>IT-01; WI-01</x:v>
-      </x:c>
-      <x:c r="L18" s="46" t="str"/>
-      <x:c r="M18" s="46" t="str"/>
-      <x:c r="N18" s="46" t="str"/>
-      <x:c r="O18" s="47"/>
+        <x:v>IT-2 (Sprint 26.1); DE-1</x:v>
+      </x:c>
+      <x:c r="L18" s="46" t="str">
+        <x:v>Committed does NOT lock scope: added DE-1 to Committed Sprint 26.1 (scope 3-&gt;4, persisted) then removed it (4-&gt;3); both succeeded. Manual status: Commit/Accept Iteration buttons exist, but committing a 2nd iteration is blocked - Another iteration is already committed for this project (single Committed per project, not in business define; DEV-022). DE-1 restored to No iteration.</x:v>
+      </x:c>
+      <x:c r="M18" s="46" t="str">
+        <x:v>DEV-022</x:v>
+      </x:c>
+      <x:c r="N18" s="46" t="str">
+        <x:v>notes/E2E-11-13-STATUS-ITERATION.md</x:v>
+      </x:c>
+      <x:c r="O18" s="47" t="n">
+        <x:v>46223</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="O19" s="48"/>
@@ -1975,14 +2019,14 @@
         <x:v>Planning</x:v>
       </x:c>
       <x:c r="J6" s="46" t="str">
-        <x:v>Planning</x:v>
+        <x:v>Wiped (reseed)</x:v>
       </x:c>
       <x:c r="K6" s="46" t="str"/>
       <x:c r="L6" s="46" t="str">
         <x:v>Keep</x:v>
       </x:c>
       <x:c r="M6" s="46" t="str">
-        <x:v>Created once and persisted after reload</x:v>
+        <x:v>Created once and persisted after reload | Wiped on 2026-07-20 DevInt reseed (iterations now only Sprint 26.1/26.2)</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="54" customHeight="1">
@@ -2014,7 +2058,7 @@
         <x:v>Planning</x:v>
       </x:c>
       <x:c r="J7" s="46" t="str">
-        <x:v>Planning</x:v>
+        <x:v>Wiped (reseed)</x:v>
       </x:c>
       <x:c r="K7" s="46" t="str">
         <x:v>MS-01</x:v>
@@ -2023,7 +2067,7 @@
         <x:v>Keep</x:v>
       </x:c>
       <x:c r="M7" s="46" t="str">
-        <x:v>Created once and persisted; earlier start</x:v>
+        <x:v>Created once and persisted; earlier start | Wiped on 2026-07-20 DevInt reseed</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="54" customHeight="1">
@@ -2055,7 +2099,7 @@
         <x:v>Planning</x:v>
       </x:c>
       <x:c r="J8" s="46" t="str">
-        <x:v>Planning</x:v>
+        <x:v>Wiped (reseed)</x:v>
       </x:c>
       <x:c r="K8" s="46" t="str">
         <x:v>MS-01</x:v>
@@ -2064,7 +2108,7 @@
         <x:v>Keep</x:v>
       </x:c>
       <x:c r="M8" s="46" t="str">
-        <x:v>Created once and persisted; later end</x:v>
+        <x:v>Created once and persisted; later end | Wiped on 2026-07-20 DevInt reseed</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
@@ -2096,7 +2140,7 @@
         <x:v>Planned</x:v>
       </x:c>
       <x:c r="J9" s="46" t="str">
-        <x:v>Planned; actual dates blank</x:v>
+        <x:v>Wiped (reseed)</x:v>
       </x:c>
       <x:c r="K9" s="46" t="str">
         <x:v>REL-01; REL-02 not selectable</x:v>
@@ -2105,7 +2149,7 @@
         <x:v>Keep</x:v>
       </x:c>
       <x:c r="M9" s="46" t="str">
-        <x:v>Standalone creation persisted; expected dates shown here are blocked derivation targets</x:v>
+        <x:v>Standalone creation persisted | Wiped on 2026-07-20 DevInt reseed</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
@@ -2119,7 +2163,7 @@
         <x:v>BA-E2E-20260720 Story / existing surrogate</x:v>
       </x:c>
       <x:c r="D10" s="46" t="str">
-        <x:v>US-12</x:v>
+        <x:v>US-9</x:v>
       </x:c>
       <x:c r="E10" s="46" t="str">
         <x:v>NXP</x:v>
@@ -2133,7 +2177,7 @@
         <x:v>Defined (existing)</x:v>
       </x:c>
       <x:c r="J10" s="46" t="str">
-        <x:v>Defined; Iteration and Release assigned</x:v>
+        <x:v>Completed (Schedule); Flow Defined; Sprint 26.2</x:v>
       </x:c>
       <x:c r="K10" s="46" t="str">
         <x:v>IT-01; REL-02; planned MS-01</x:v>
@@ -2142,7 +2186,7 @@
         <x:v>Keep</x:v>
       </x:c>
       <x:c r="M10" s="46" t="str">
-        <x:v>Existing US-12 is the surrogate. IT-5 and Release B persisted; Work Item Detail has no Milestone field.</x:v>
+        <x:v>Reseed 2026-07-20: surrogate is now US-9 (was US-12). Assigned Sprint 26.2; Schedule Completed via Task roll-up, Flow stayed Defined; no Milestone field.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
@@ -2156,7 +2200,7 @@
         <x:v>BA-E2E-20260720 Task A</x:v>
       </x:c>
       <x:c r="D11" s="46" t="str">
-        <x:v>TA-8</x:v>
+        <x:v>TA-6</x:v>
       </x:c>
       <x:c r="E11" s="46" t="str">
         <x:v>NXP inherited</x:v>
@@ -2170,7 +2214,7 @@
         <x:v>Defined</x:v>
       </x:c>
       <x:c r="J11" s="46" t="str">
-        <x:v>Defined</x:v>
+        <x:v>In Progress</x:v>
       </x:c>
       <x:c r="K11" s="46" t="str">
         <x:v>WI-01 / US-12</x:v>
@@ -2179,7 +2223,7 @@
         <x:v>Keep</x:v>
       </x:c>
       <x:c r="M11" s="46" t="str">
-        <x:v>Created with editable Estimate 4; To Do/Actuals blank; persisted after reload</x:v>
+        <x:v>Reseed 2026-07-20: now TA-6 under US-9. In Progress; To Do 0, Actual 2h (Time Logs). Estimate blank.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
@@ -2193,7 +2237,7 @@
         <x:v>BA-E2E-20260720 Task B</x:v>
       </x:c>
       <x:c r="D12" s="46" t="str">
-        <x:v>TA-9</x:v>
+        <x:v>TA-7</x:v>
       </x:c>
       <x:c r="E12" s="46" t="str">
         <x:v>NXP inherited</x:v>
@@ -2207,7 +2251,7 @@
         <x:v>Defined</x:v>
       </x:c>
       <x:c r="J12" s="46" t="str">
-        <x:v>Defined</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="K12" s="46" t="str">
         <x:v>WI-01 / US-12</x:v>
@@ -2216,7 +2260,7 @@
         <x:v>Keep</x:v>
       </x:c>
       <x:c r="M12" s="46" t="str">
-        <x:v>Created with editable Estimate 2; To Do/Actuals blank; persisted after reload</x:v>
+        <x:v>Reseed 2026-07-20: now TA-7 under US-9. Completed; Estimate 4, To Do 0, Actual 0.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -3426,101 +3470,261 @@
         <x:v>Resume at E2E-08; do not recreate TA-8 or TA-9</x:v>
       </x:c>
     </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="46"/>
-      <x:c r="B36" s="46"/>
-      <x:c r="C36" s="50"/>
-      <x:c r="D36" s="46"/>
-      <x:c r="E36" s="46"/>
-      <x:c r="F36" s="46"/>
-      <x:c r="G36" s="46"/>
-      <x:c r="H36" s="46"/>
-      <x:c r="I36" s="46"/>
-      <x:c r="J36" s="46"/>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="46"/>
-      <x:c r="B37" s="46"/>
-      <x:c r="C37" s="50"/>
-      <x:c r="D37" s="46"/>
-      <x:c r="E37" s="46"/>
-      <x:c r="F37" s="46"/>
-      <x:c r="G37" s="46"/>
-      <x:c r="H37" s="46"/>
-      <x:c r="I37" s="46"/>
-      <x:c r="J37" s="46"/>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="46"/>
-      <x:c r="B38" s="46"/>
-      <x:c r="C38" s="50"/>
-      <x:c r="D38" s="46"/>
-      <x:c r="E38" s="46"/>
-      <x:c r="F38" s="46"/>
-      <x:c r="G38" s="46"/>
-      <x:c r="H38" s="46"/>
-      <x:c r="I38" s="46"/>
-      <x:c r="J38" s="46"/>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="46"/>
-      <x:c r="B39" s="46"/>
-      <x:c r="C39" s="50"/>
-      <x:c r="D39" s="46"/>
-      <x:c r="E39" s="46"/>
-      <x:c r="F39" s="46"/>
-      <x:c r="G39" s="46"/>
-      <x:c r="H39" s="46"/>
-      <x:c r="I39" s="46"/>
-      <x:c r="J39" s="46"/>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="46"/>
-      <x:c r="B40" s="46"/>
-      <x:c r="C40" s="50"/>
-      <x:c r="D40" s="46"/>
-      <x:c r="E40" s="46"/>
-      <x:c r="F40" s="46"/>
-      <x:c r="G40" s="46"/>
-      <x:c r="H40" s="46"/>
-      <x:c r="I40" s="46"/>
-      <x:c r="J40" s="46"/>
-    </x:row>
-    <x:row r="41">
-      <x:c r="A41" s="46"/>
-      <x:c r="B41" s="46"/>
-      <x:c r="C41" s="50"/>
-      <x:c r="D41" s="46"/>
-      <x:c r="E41" s="46"/>
-      <x:c r="F41" s="46"/>
-      <x:c r="G41" s="46"/>
-      <x:c r="H41" s="46"/>
-      <x:c r="I41" s="46"/>
-      <x:c r="J41" s="46"/>
-    </x:row>
-    <x:row r="42">
-      <x:c r="A42" s="46"/>
-      <x:c r="B42" s="46"/>
-      <x:c r="C42" s="50"/>
-      <x:c r="D42" s="46"/>
-      <x:c r="E42" s="46"/>
-      <x:c r="F42" s="46"/>
-      <x:c r="G42" s="46"/>
-      <x:c r="H42" s="46"/>
-      <x:c r="I42" s="46"/>
-      <x:c r="J42" s="46"/>
-    </x:row>
-    <x:row r="43">
-      <x:c r="A43" s="46"/>
-      <x:c r="B43" s="46"/>
-      <x:c r="C43" s="50"/>
-      <x:c r="D43" s="46"/>
-      <x:c r="E43" s="46"/>
-      <x:c r="F43" s="46"/>
-      <x:c r="G43" s="46"/>
-      <x:c r="H43" s="46"/>
-      <x:c r="I43" s="46"/>
-      <x:c r="J43" s="46"/>
+    <x:row r="36" ht="72" customHeight="1">
+      <x:c r="A36" s="46" t="str">
+        <x:v>EXEC-032</x:v>
+      </x:c>
+      <x:c r="B36" s="46" t="str">
+        <x:v>E2E-08</x:v>
+      </x:c>
+      <x:c r="C36" s="50" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D36" s="46" t="str">
+        <x:v>Work Item Detail &gt; Tasks / US-9</x:v>
+      </x:c>
+      <x:c r="E36" s="46" t="str">
+        <x:v>Recreate controlled Tasks after reseed</x:v>
+      </x:c>
+      <x:c r="F36" s="46" t="str">
+        <x:v>Two child Tasks created once with default Defined and inherited context</x:v>
+      </x:c>
+      <x:c r="G36" s="46" t="str">
+        <x:v>TA-6 and TA-7 created once under US-9, default Defined, NXP / no team; TA-7 accepted an independent Estimate 4 with blank To Do/Actual</x:v>
+      </x:c>
+      <x:c r="H36" s="46" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I36" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="J36" s="46" t="str">
+        <x:v>Reseed wiped TA-8/TA-9; tab badge still shows 0 (DEV-012)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="72" customHeight="1">
+      <x:c r="A37" s="46" t="str">
+        <x:v>EXEC-033</x:v>
+      </x:c>
+      <x:c r="B37" s="46" t="str">
+        <x:v>E2E-08</x:v>
+      </x:c>
+      <x:c r="C37" s="50" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D37" s="46" t="str">
+        <x:v>Task Detail / TA-6</x:v>
+      </x:c>
+      <x:c r="E37" s="46" t="str">
+        <x:v>Set To Do=3 and log Actual=2h; observe Estimate</x:v>
+      </x:c>
+      <x:c r="F37" s="46" t="str">
+        <x:v>Estimate becomes read-only 5 (To Do + Actuals)</x:v>
+      </x:c>
+      <x:c r="G37" s="46" t="str">
+        <x:v>Estimate stayed blank; US-9 roll-up Estimate 4 != To Do 3 + Actual 2 = 5; Actual entered via Time Logs entry-sum</x:v>
+      </x:c>
+      <x:c r="H37" s="46" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="I37" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="J37" s="46" t="str">
+        <x:v>DEV-013 / DEV-015 reconfirmed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="72" customHeight="1">
+      <x:c r="A38" s="46" t="str">
+        <x:v>EXEC-034</x:v>
+      </x:c>
+      <x:c r="B38" s="46" t="str">
+        <x:v>E2E-09</x:v>
+      </x:c>
+      <x:c r="C38" s="50" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D38" s="46" t="str">
+        <x:v>Task Detail / TA-6</x:v>
+      </x:c>
+      <x:c r="E38" s="46" t="str">
+        <x:v>Complete only TA-6 (1 of 2)</x:v>
+      </x:c>
+      <x:c r="F38" s="46" t="str">
+        <x:v>Parent stays not Completed</x:v>
+      </x:c>
+      <x:c r="G38" s="46" t="str">
+        <x:v>US-9 stayed Defined; completing TA-6 also zeroed its To Do</x:v>
+      </x:c>
+      <x:c r="H38" s="46" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I38" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="J38" s="46" t="str">
+        <x:v>Partial-completion guard correct</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="72" customHeight="1">
+      <x:c r="A39" s="46" t="str">
+        <x:v>EXEC-035</x:v>
+      </x:c>
+      <x:c r="B39" s="46" t="str">
+        <x:v>E2E-09</x:v>
+      </x:c>
+      <x:c r="C39" s="50" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D39" s="46" t="str">
+        <x:v>Task Detail / TA-7</x:v>
+      </x:c>
+      <x:c r="E39" s="46" t="str">
+        <x:v>Complete TA-7 so all child Tasks are Completed</x:v>
+      </x:c>
+      <x:c r="F39" s="46" t="str">
+        <x:v>Parent Schedule and Flow both auto-change to Completed</x:v>
+      </x:c>
+      <x:c r="G39" s="46" t="str">
+        <x:v>US-9 Schedule State auto-Completed; Flow State stayed Defined (no mirror)</x:v>
+      </x:c>
+      <x:c r="H39" s="46" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="I39" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="J39" s="46" t="str">
+        <x:v>DEV-017</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="72" customHeight="1">
+      <x:c r="A40" s="46" t="str">
+        <x:v>EXEC-036</x:v>
+      </x:c>
+      <x:c r="B40" s="46" t="str">
+        <x:v>E2E-10</x:v>
+      </x:c>
+      <x:c r="C40" s="50" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D40" s="46" t="str">
+        <x:v>Task Detail / TA-6</x:v>
+      </x:c>
+      <x:c r="E40" s="46" t="str">
+        <x:v>Reopen TA-6 to In Progress</x:v>
+      </x:c>
+      <x:c r="F40" s="46" t="str">
+        <x:v>Parent auto-moves to In-Progress</x:v>
+      </x:c>
+      <x:c r="G40" s="46" t="str">
+        <x:v>TA-6 persisted In Progress after reload; US-9 stayed Completed, no roll-back</x:v>
+      </x:c>
+      <x:c r="H40" s="46" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="I40" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="J40" s="46" t="str">
+        <x:v>DEV-018; auto roll-up one-way</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41" ht="72" customHeight="1">
+      <x:c r="A41" s="46" t="str">
+        <x:v>EXEC-037</x:v>
+      </x:c>
+      <x:c r="B41" s="46" t="str">
+        <x:v>E2E-05</x:v>
+      </x:c>
+      <x:c r="C41" s="50" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D41" s="46" t="str">
+        <x:v>Work Item Detail / US-9</x:v>
+      </x:c>
+      <x:c r="E41" s="46" t="str">
+        <x:v>Assign US-9 to Sprint 26.2 (post-reseed retest)</x:v>
+      </x:c>
+      <x:c r="F41" s="46" t="str">
+        <x:v>Assignment persists and same ID appears in Iteration Status</x:v>
+      </x:c>
+      <x:c r="G41" s="46" t="str">
+        <x:v>US-9 assigned to Sprint 26.2; appears once in Iteration Status Sprint 26.2 with Schedule State C</x:v>
+      </x:c>
+      <x:c r="H41" s="46" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="I41" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="J41" s="46" t="str">
+        <x:v>Cross-screen identity now testable after reseed</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="72" customHeight="1">
+      <x:c r="A42" s="46" t="str">
+        <x:v>EXEC-038</x:v>
+      </x:c>
+      <x:c r="B42" s="46" t="str">
+        <x:v>E2E-05</x:v>
+      </x:c>
+      <x:c r="C42" s="50" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D42" s="46" t="str">
+        <x:v>Track &gt; Iteration Status / Sprint 26.2</x:v>
+      </x:c>
+      <x:c r="E42" s="46" t="str">
+        <x:v>Verify US-9 roll-up metrics</x:v>
+      </x:c>
+      <x:c r="F42" s="46" t="str">
+        <x:v>Task Est/To Do totals roll up; active count reflects not-Completed tasks</x:v>
+      </x:c>
+      <x:c r="G42" s="46" t="str">
+        <x:v>Totals Task Est 4 / To Do 0 correct, but US-9 shows Tasks 100% and top tile 0 Active Tasks though TA-6 is In Progress</x:v>
+      </x:c>
+      <x:c r="H42" s="46" t="str">
+        <x:v>Failed</x:v>
+      </x:c>
+      <x:c r="I42" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="J42" s="46" t="str">
+        <x:v>DEV-019</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43" ht="72" customHeight="1">
+      <x:c r="A43" s="46" t="str">
+        <x:v>EXEC-039</x:v>
+      </x:c>
+      <x:c r="B43" s="46" t="str">
+        <x:v>E2E-05</x:v>
+      </x:c>
+      <x:c r="C43" s="50" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D43" s="46" t="str">
+        <x:v>Track &gt; Team Status / Sprint 26.2</x:v>
+      </x:c>
+      <x:c r="E43" s="46" t="str">
+        <x:v>Verify per-owner task roll-up</x:v>
+      </x:c>
+      <x:c r="F43" s="46" t="str">
+        <x:v>Same child Tasks roll to owner with correct counts</x:v>
+      </x:c>
+      <x:c r="G43" s="46" t="str">
+        <x:v>Alice Developer (2 Tasks) 50%, Estimate 4 / To Do 0 / Actuals 2 - state-based 50% disagrees with Iteration Status 100%</x:v>
+      </x:c>
+      <x:c r="H43" s="46" t="str">
+        <x:v>Partial</x:v>
+      </x:c>
+      <x:c r="I43" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="J43" s="46" t="str">
+        <x:v>Identity roll-up correct; metric inconsistent (DEV-019)</x:v>
+      </x:c>
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="46"/>
@@ -4951,125 +5155,333 @@
         <x:v>BA confirmed inline editing is required on 2026-07-20</x:v>
       </x:c>
     </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="46"/>
-      <x:c r="B21" s="46"/>
-      <x:c r="C21" s="46"/>
-      <x:c r="D21" s="46"/>
-      <x:c r="E21" s="46"/>
-      <x:c r="F21" s="46"/>
-      <x:c r="G21" s="46"/>
-      <x:c r="H21" s="46"/>
-      <x:c r="I21" s="46"/>
-      <x:c r="J21" s="46"/>
-      <x:c r="K21" s="46"/>
-      <x:c r="L21" s="46"/>
-      <x:c r="M21" s="46"/>
-    </x:row>
-    <x:row r="22">
-      <x:c r="A22" s="46"/>
-      <x:c r="B22" s="46"/>
-      <x:c r="C22" s="46"/>
-      <x:c r="D22" s="46"/>
-      <x:c r="E22" s="46"/>
-      <x:c r="F22" s="46"/>
-      <x:c r="G22" s="46"/>
-      <x:c r="H22" s="46"/>
-      <x:c r="I22" s="46"/>
-      <x:c r="J22" s="46"/>
-      <x:c r="K22" s="46"/>
-      <x:c r="L22" s="46"/>
-      <x:c r="M22" s="46"/>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="46"/>
-      <x:c r="B23" s="46"/>
-      <x:c r="C23" s="46"/>
-      <x:c r="D23" s="46"/>
-      <x:c r="E23" s="46"/>
-      <x:c r="F23" s="46"/>
-      <x:c r="G23" s="46"/>
-      <x:c r="H23" s="46"/>
-      <x:c r="I23" s="46"/>
-      <x:c r="J23" s="46"/>
-      <x:c r="K23" s="46"/>
-      <x:c r="L23" s="46"/>
-      <x:c r="M23" s="46"/>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="46"/>
-      <x:c r="B24" s="46"/>
-      <x:c r="C24" s="46"/>
-      <x:c r="D24" s="46"/>
-      <x:c r="E24" s="46"/>
-      <x:c r="F24" s="46"/>
-      <x:c r="G24" s="46"/>
-      <x:c r="H24" s="46"/>
-      <x:c r="I24" s="46"/>
-      <x:c r="J24" s="46"/>
-      <x:c r="K24" s="46"/>
-      <x:c r="L24" s="46"/>
-      <x:c r="M24" s="46"/>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="46"/>
-      <x:c r="B25" s="46"/>
-      <x:c r="C25" s="46"/>
-      <x:c r="D25" s="46"/>
-      <x:c r="E25" s="46"/>
-      <x:c r="F25" s="46"/>
-      <x:c r="G25" s="46"/>
-      <x:c r="H25" s="46"/>
-      <x:c r="I25" s="46"/>
-      <x:c r="J25" s="46"/>
-      <x:c r="K25" s="46"/>
-      <x:c r="L25" s="46"/>
-      <x:c r="M25" s="46"/>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="46"/>
-      <x:c r="B26" s="46"/>
-      <x:c r="C26" s="46"/>
-      <x:c r="D26" s="46"/>
-      <x:c r="E26" s="46"/>
-      <x:c r="F26" s="46"/>
-      <x:c r="G26" s="46"/>
-      <x:c r="H26" s="46"/>
-      <x:c r="I26" s="46"/>
-      <x:c r="J26" s="46"/>
-      <x:c r="K26" s="46"/>
-      <x:c r="L26" s="46"/>
-      <x:c r="M26" s="46"/>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="46"/>
-      <x:c r="B27" s="46"/>
-      <x:c r="C27" s="46"/>
-      <x:c r="D27" s="46"/>
-      <x:c r="E27" s="46"/>
-      <x:c r="F27" s="46"/>
-      <x:c r="G27" s="46"/>
-      <x:c r="H27" s="46"/>
-      <x:c r="I27" s="46"/>
-      <x:c r="J27" s="46"/>
-      <x:c r="K27" s="46"/>
-      <x:c r="L27" s="46"/>
-      <x:c r="M27" s="46"/>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="46"/>
-      <x:c r="B28" s="46"/>
-      <x:c r="C28" s="46"/>
-      <x:c r="D28" s="46"/>
-      <x:c r="E28" s="46"/>
-      <x:c r="F28" s="46"/>
-      <x:c r="G28" s="46"/>
-      <x:c r="H28" s="46"/>
-      <x:c r="I28" s="46"/>
-      <x:c r="J28" s="46"/>
-      <x:c r="K28" s="46"/>
-      <x:c r="L28" s="46"/>
-      <x:c r="M28" s="46"/>
+    <x:row r="21" ht="72" customHeight="1">
+      <x:c r="A21" s="46" t="str">
+        <x:v>DEV-015</x:v>
+      </x:c>
+      <x:c r="B21" s="46" t="str">
+        <x:v>E2E-08</x:v>
+      </x:c>
+      <x:c r="C21" s="46" t="str">
+        <x:v>Task time / Actual model</x:v>
+      </x:c>
+      <x:c r="D21" s="46" t="str">
+        <x:v>Estimate is read-only and equals To Do + Actuals; Actual is a manual value per confirmed Phase 1</x:v>
+      </x:c>
+      <x:c r="E21" s="46" t="str">
+        <x:v>Estimate stays an independent editable field and does not derive (roll-up Estimate 4 != To Do 3 + Actual 2 = 5). Actual is captured as a Time Logs entry-sum, and completing a Task silently zeroes its To Do.</x:v>
+      </x:c>
+      <x:c r="F21" s="46" t="str">
+        <x:v>Business Contract</x:v>
+      </x:c>
+      <x:c r="G21" s="46" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H21" s="46" t="str">
+        <x:v>Make Estimate read-only and always derive To Do + Actuals at Task, roll-up and Add Task modal; capture Actual as a manual input as in the mockup (replace the Time Logs entry-sum); do not auto-zero To Do when a Task is completed.</x:v>
+      </x:c>
+      <x:c r="I21" s="46" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="J21" s="46" t="str">
+        <x:v>Dev / BA / Docs</x:v>
+      </x:c>
+      <x:c r="K21" s="46" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L21" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="M21" s="46" t="str">
+        <x:v>BA 2026-07-20: Estimate derived read-only; Actual is a MANUAL input as in the mockup (not the Time Logs entry-sum); completing a Task must not silently zero To Do. Reconfirms DEV-013 / DOC-002.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="72" customHeight="1">
+      <x:c r="A22" s="46" t="str">
+        <x:v>DEV-016</x:v>
+      </x:c>
+      <x:c r="B22" s="46" t="str">
+        <x:v>E2E-08; E2E-09; E2E-10</x:v>
+      </x:c>
+      <x:c r="C22" s="46" t="str">
+        <x:v>Task Detail state model</x:v>
+      </x:c>
+      <x:c r="D22" s="46" t="str">
+        <x:v>A Task has a single Task State (Defined, In-Progress, Completed) per BR-TASK-01</x:v>
+      </x:c>
+      <x:c r="E22" s="46" t="str">
+        <x:v>Task Detail exposes Schedule State (six buttons) plus Flow State (four-option dropdown) - the Story/Defect model, not a single Task State. Label uses In Progress, not In-Progress.</x:v>
+      </x:c>
+      <x:c r="F22" s="46" t="str">
+        <x:v>UI / Business</x:v>
+      </x:c>
+      <x:c r="G22" s="46" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H22" s="46" t="str">
+        <x:v>Replace Schedule + Flow State on Task Detail/Dashboard with a single Task State control using the exact catalog Defined/In-Progress/Completed.</x:v>
+      </x:c>
+      <x:c r="I22" s="46" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="J22" s="46" t="str">
+        <x:v>Dev</x:v>
+      </x:c>
+      <x:c r="K22" s="46" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L22" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="M22" s="46" t="str">
+        <x:v>BA confirmed 2026-07-20: remove Schedule + Flow State on Task; Task Detail/Dashboard design must match the mockup single Task State (Defined/In-Progress/Completed).</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="72" customHeight="1">
+      <x:c r="A23" s="46" t="str">
+        <x:v>DEV-017</x:v>
+      </x:c>
+      <x:c r="B23" s="46" t="str">
+        <x:v>E2E-09</x:v>
+      </x:c>
+      <x:c r="C23" s="46" t="str">
+        <x:v>Parent roll-up on all-Tasks-Completed</x:v>
+      </x:c>
+      <x:c r="D23" s="46" t="str">
+        <x:v>When all child Tasks are Completed the parent Schedule State AND Flow State both change to Completed and mirror (BR-WI-01; TASK-FR-016)</x:v>
+      </x:c>
+      <x:c r="E23" s="46" t="str">
+        <x:v>US-9 Schedule State auto-changed to Completed, but Flow State stayed Defined; the two fields did not mirror.</x:v>
+      </x:c>
+      <x:c r="F23" s="46" t="str">
+        <x:v>Business Contract</x:v>
+      </x:c>
+      <x:c r="G23" s="46" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H23" s="46" t="str">
+        <x:v>On auto roll-up set both Schedule and Flow State to Completed; enforce Schedule &lt;-&gt; Flow mirroring in both directions generally.</x:v>
+      </x:c>
+      <x:c r="I23" s="46" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="J23" s="46" t="str">
+        <x:v>Dev</x:v>
+      </x:c>
+      <x:c r="K23" s="46" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L23" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="M23" s="46" t="str">
+        <x:v>Auto-complete direction works; only the mirror is missing. BA confirmed 2026-07-20.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="72" customHeight="1">
+      <x:c r="A24" s="46" t="str">
+        <x:v>DEV-018</x:v>
+      </x:c>
+      <x:c r="B24" s="46" t="str">
+        <x:v>E2E-10</x:v>
+      </x:c>
+      <x:c r="C24" s="46" t="str">
+        <x:v>Parent roll-up on Task reopen</x:v>
+      </x:c>
+      <x:c r="D24" s="46" t="str">
+        <x:v>Reopening any child Task after all were Completed auto-moves the parent back to In-Progress (BR-TASK-02); manual control remains</x:v>
+      </x:c>
+      <x:c r="E24" s="46" t="str">
+        <x:v>Reopened TA-6 to In Progress and it persisted, but US-9 stayed Completed; the parent did not roll back.</x:v>
+      </x:c>
+      <x:c r="F24" s="46" t="str">
+        <x:v>Missing Function</x:v>
+      </x:c>
+      <x:c r="G24" s="46" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H24" s="46" t="str">
+        <x:v>Implement the reverse roll-up so reopening a child Task sets the parent to In-Progress; keep manual override.</x:v>
+      </x:c>
+      <x:c r="I24" s="46" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="J24" s="46" t="str">
+        <x:v>Dev</x:v>
+      </x:c>
+      <x:c r="K24" s="46" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L24" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="M24" s="46" t="str">
+        <x:v>Auto roll-up is currently one-way only. BA confirmed 2026-07-20.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="72" customHeight="1">
+      <x:c r="A25" s="46" t="str">
+        <x:v>DEV-019</x:v>
+      </x:c>
+      <x:c r="B25" s="46" t="str">
+        <x:v>E2E-05</x:v>
+      </x:c>
+      <x:c r="C25" s="46" t="str">
+        <x:v>Iteration Status vs Team Status task metric</x:v>
+      </x:c>
+      <x:c r="D25" s="46" t="str">
+        <x:v>Iteration Status header metrics per BA: Planned Velocity is deferred to Phase 5 (not defined yet); Iteration End counts days; Accepted is the percent of US/DE that are Accepted. Task active-count and Task percent use child Task State (not Completed) and agree with Team Status.</x:v>
+      </x:c>
+      <x:c r="E25" s="46" t="str">
+        <x:v>For US-9 (TA-6 In Progress, TA-7 Completed) Team Status shows Alice 2 Tasks 50% (state-based) but Iteration Status shows US-9 Tasks 100% and 0 Active Tasks (To-Do-based), so the two screens disagree.</x:v>
+      </x:c>
+      <x:c r="F25" s="46" t="str">
+        <x:v>Shared Data / Metric</x:v>
+      </x:c>
+      <x:c r="G25" s="46" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H25" s="46" t="str">
+        <x:v>Defer Planned Velocity to Phase 5; keep Iteration End as a day count; compute Accepted from US/DE in Accepted state; compute task active-count and Task percent from Task State consistently across Iteration Status and Team Status (not from To Do).</x:v>
+      </x:c>
+      <x:c r="I25" s="46" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="J25" s="46" t="str">
+        <x:v>Dev</x:v>
+      </x:c>
+      <x:c r="K25" s="46" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L25" s="46" t="str">
+        <x:v>notes/E2E-08-10-TASK-PROPAGATION.md</x:v>
+      </x:c>
+      <x:c r="M25" s="46" t="str">
+        <x:v>BA 2026-07-20: Planned Velocity to Phase 5; Iteration End day-count OK; Accepted counts US Accepted; task metric must be state-based and consistent with Team Status.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="72" customHeight="1">
+      <x:c r="A26" s="46" t="str">
+        <x:v>DEV-020</x:v>
+      </x:c>
+      <x:c r="B26" s="46" t="str">
+        <x:v>E2E-11</x:v>
+      </x:c>
+      <x:c r="C26" s="46" t="str">
+        <x:v>Work Item Schedule/Flow State</x:v>
+      </x:c>
+      <x:c r="D26" s="46" t="str">
+        <x:v>Schedule and Flow State both use all six values (Idea/Defined/In-Progress/Completed/Accepted/Release) and mirror bidirectionally</x:v>
+      </x:c>
+      <x:c r="E26" s="46" t="str">
+        <x:v>Flow State dropdown has only 4 options (missing Idea and Release); label In Progress not In-Progress; Schedule&lt;-&gt;Flow do not mirror in either direction (verified on US-7).</x:v>
+      </x:c>
+      <x:c r="F26" s="46" t="str">
+        <x:v>Business Contract</x:v>
+      </x:c>
+      <x:c r="G26" s="46" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="H26" s="46" t="str">
+        <x:v>Give Flow State the full six-value catalog with exact spelling In-Progress; mirror Schedule&lt;-&gt;Flow bidirectionally on every manual and automatic change; match the mockup.</x:v>
+      </x:c>
+      <x:c r="I26" s="46" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="J26" s="46" t="str">
+        <x:v>Dev</x:v>
+      </x:c>
+      <x:c r="K26" s="46" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L26" s="46" t="str">
+        <x:v>notes/E2E-11-13-STATUS-ITERATION.md</x:v>
+      </x:c>
+      <x:c r="M26" s="46" t="str">
+        <x:v>BA confirmed 2026-07-20; design must match the mockup.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="72" customHeight="1">
+      <x:c r="A27" s="46" t="str">
+        <x:v>DEV-021</x:v>
+      </x:c>
+      <x:c r="B27" s="46" t="str">
+        <x:v>E2E-12</x:v>
+      </x:c>
+      <x:c r="C27" s="46" t="str">
+        <x:v>Iteration auto-Accept</x:v>
+      </x:c>
+      <x:c r="D27" s="46" t="str">
+        <x:v>A non-empty Iteration whose assigned US/DE are all Accepted auto-changes to Accepted (BR-IT-02); manual override remains; no auto-reverse</x:v>
+      </x:c>
+      <x:c r="E27" s="46" t="str">
+        <x:v>US-7 and US-9 set to Accepted; Iteration Status Accepted = 100% (13/13) and detail Accepted 100% of committed, but Sprint 26.2 stayed Planning - no auto-transition.</x:v>
+      </x:c>
+      <x:c r="F27" s="46" t="str">
+        <x:v>Missing Function</x:v>
+      </x:c>
+      <x:c r="G27" s="46" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H27" s="46" t="str">
+        <x:v>Auto-set the Iteration State to Accepted when all scoped US/DE are Accepted; keep manual override and do not auto-reverse.</x:v>
+      </x:c>
+      <x:c r="I27" s="46" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="J27" s="46" t="str">
+        <x:v>Dev</x:v>
+      </x:c>
+      <x:c r="K27" s="46" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L27" s="46" t="str">
+        <x:v>notes/E2E-11-13-STATUS-ITERATION.md</x:v>
+      </x:c>
+      <x:c r="M27" s="46" t="str">
+        <x:v>BA confirmed 2026-07-20: per SRS/mockup the Iteration must auto-change to Accepted when all US/DE are Accepted and must remain manually editable. Accepted metric is already correct; only the auto state transition is missing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="72" customHeight="1">
+      <x:c r="A28" s="46" t="str">
+        <x:v>DEV-022</x:v>
+      </x:c>
+      <x:c r="B28" s="46" t="str">
+        <x:v>E2E-13</x:v>
+      </x:c>
+      <x:c r="C28" s="46" t="str">
+        <x:v>Iteration commit restriction</x:v>
+      </x:c>
+      <x:c r="D28" s="46" t="str">
+        <x:v>The business define does not limit the number of Committed iterations per project; the user retains manual status control</x:v>
+      </x:c>
+      <x:c r="E28" s="46" t="str">
+        <x:v>Committing a second iteration is blocked with Another iteration is already committed for this project.</x:v>
+      </x:c>
+      <x:c r="F28" s="46" t="str">
+        <x:v>Business / Validation</x:v>
+      </x:c>
+      <x:c r="G28" s="46" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="H28" s="46" t="str">
+        <x:v>Allow multiple Committed iterations per project (remove the single-committed restriction).</x:v>
+      </x:c>
+      <x:c r="I28" s="46" t="str">
+        <x:v>Confirmed</x:v>
+      </x:c>
+      <x:c r="J28" s="46" t="str">
+        <x:v>Dev</x:v>
+      </x:c>
+      <x:c r="K28" s="46" t="str">
+        <x:v>Not Run</x:v>
+      </x:c>
+      <x:c r="L28" s="46" t="str">
+        <x:v>notes/E2E-11-13-STATUS-ITERATION.md</x:v>
+      </x:c>
+      <x:c r="M28" s="46" t="str">
+        <x:v>BA confirmed 2026-07-20 that multiple Committed iterations per project are allowed.</x:v>
+      </x:c>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="46"/>

</xml_diff>